<commit_message>
v2 measurements: per-image summary stats (mean/median/SD) over interior lacunae (v2-raw, pre-validation)
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/results/count/542_WT__2_z06c1-2/measurements.xlsx
+++ b/results/count/542_WT__2_z06c1-2/measurements.xlsx
@@ -414,7 +414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D2"/>
+  <dimension ref="A1:F11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -452,6 +452,189 @@
         <v>3</v>
       </c>
       <c r="D2" t="n">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>v2-raw / pre-validation -- stats below over interior (on_border=False) lacunae only</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>metric</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>mean</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>median</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>sd</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>units</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>n</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>area</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>2004.4118</v>
+      </c>
+      <c r="C6" t="n">
+        <v>1720</v>
+      </c>
+      <c r="D6" t="n">
+        <v>1474.8632</v>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>px</t>
+        </is>
+      </c>
+      <c r="F6" t="n">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>major_axis_length</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>88.87260000000001</v>
+      </c>
+      <c r="C7" t="n">
+        <v>77.8309</v>
+      </c>
+      <c r="D7" t="n">
+        <v>44.7578</v>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>px</t>
+        </is>
+      </c>
+      <c r="F7" t="n">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>minor_axis_length</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>29.1534</v>
+      </c>
+      <c r="C8" t="n">
+        <v>29.6128</v>
+      </c>
+      <c r="D8" t="n">
+        <v>10.3063</v>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>px</t>
+        </is>
+      </c>
+      <c r="F8" t="n">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>aspect_ratio</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>3.1061</v>
+      </c>
+      <c r="C9" t="n">
+        <v>3.0469</v>
+      </c>
+      <c r="D9" t="n">
+        <v>1.2971</v>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>unitless</t>
+        </is>
+      </c>
+      <c r="F9" t="n">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>eccentricity</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
+        <v>0.9105</v>
+      </c>
+      <c r="C10" t="n">
+        <v>0.9446</v>
+      </c>
+      <c r="D10" t="n">
+        <v>0.0696</v>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>unitless</t>
+        </is>
+      </c>
+      <c r="F10" t="n">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>solidity</t>
+        </is>
+      </c>
+      <c r="B11" t="n">
+        <v>0.7736</v>
+      </c>
+      <c r="C11" t="n">
+        <v>0.7956</v>
+      </c>
+      <c r="D11" t="n">
+        <v>0.1245</v>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>unitless</t>
+        </is>
+      </c>
+      <c r="F11" t="n">
         <v>17</v>
       </c>
     </row>

</xml_diff>